<commit_message>
add final test report and summary
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="120">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -378,9 +378,6 @@
   </si>
   <si>
     <t>Payment recorded successfully, invoice status updated accordingly</t>
-  </si>
-  <si>
-    <t>User created successfully with empty fields, no validation applied</t>
   </si>
   <si>
     <t>Tenant created successfully, new tenant returned with id = X and correct data</t>
@@ -854,13 +851,13 @@
         <v>44</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>118</v>
+      <c r="I3" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>56</v>
@@ -1000,7 +997,7 @@
         <v>63</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>47</v>
@@ -1012,7 +1009,7 @@
         <v>53</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>65</v>

</xml_diff>